<commit_message>
Allow new-customer submit without CI, NAR1, or registry extracts.
Sales plan plus Contact 1 ID and a Sales colleague selection are enough to apply; typed authorized signature is no longer required.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/KIRII_New_Customer_Parts2-4_Questionnaire_SAMPLE.xlsx
+++ b/public/templates/KIRII_New_Customer_Parts2-4_Questionnaire_SAMPLE.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="315">
   <si>
     <t>HK District / 香港分區</t>
   </si>
@@ -600,97 +600,100 @@
     <t>contacts.0.idNumber</t>
   </si>
   <si>
-    <t>Contact 1 / 聯絡人 1 - ID Number / 身分證號碼</t>
+    <t>Contact 1 / 聯絡人 1 - ID Number / 身分證號碼 *</t>
   </si>
   <si>
     <t>A123456(7)</t>
   </si>
   <si>
+    <t>Required. As shown on ID copy / 必須。與身分證副本一致</t>
+  </si>
+  <si>
+    <t>contacts.0.title</t>
+  </si>
+  <si>
+    <t>Contact 1 / 聯絡人 1 - Title / 職位</t>
+  </si>
+  <si>
+    <t>Purchasing Manager</t>
+  </si>
+  <si>
+    <t>contacts.0.email</t>
+  </si>
+  <si>
+    <t>Contact 1 / 聯絡人 1 - Email / 電郵</t>
+  </si>
+  <si>
+    <t>john.wong@apex-trading-demo.hk</t>
+  </si>
+  <si>
+    <t>contacts.0.phoneCountryCode</t>
+  </si>
+  <si>
+    <t>Contact 1 / 聯絡人 1 - Phone Country Code / 電話區號</t>
+  </si>
+  <si>
+    <t>+852</t>
+  </si>
+  <si>
+    <t>e.g. +852</t>
+  </si>
+  <si>
+    <t>contacts.0.phone</t>
+  </si>
+  <si>
+    <t>Contact 1 / 聯絡人 1 - Phone / 電話</t>
+  </si>
+  <si>
+    <t>9123 4567</t>
+  </si>
+  <si>
+    <t>contacts.1.nameEnFirst</t>
+  </si>
+  <si>
+    <t>Contact 2 / 聯絡人 2 - Given Name (English) / 英文名 *</t>
+  </si>
+  <si>
+    <t>Mary</t>
+  </si>
+  <si>
+    <t>contacts.1.nameEnMiddle</t>
+  </si>
+  <si>
+    <t>Contact 2 / 聯絡人 2 - Middle Name (English) / 英文中間名</t>
+  </si>
+  <si>
+    <t>Ann</t>
+  </si>
+  <si>
+    <t>contacts.1.nameEnLast</t>
+  </si>
+  <si>
+    <t>Contact 2 / 聯絡人 2 - Surname (English) / 英文姓氏 *</t>
+  </si>
+  <si>
+    <t>Cheung</t>
+  </si>
+  <si>
+    <t>contacts.1.nameZh</t>
+  </si>
+  <si>
+    <t>Contact 2 / 聯絡人 2 - Full Name (Chinese) / 中文姓名全名 *</t>
+  </si>
+  <si>
+    <t>張麗珍</t>
+  </si>
+  <si>
+    <t>contacts.1.idNumber</t>
+  </si>
+  <si>
+    <t>Contact 2 / 聯絡人 2 - ID Number / 身分證號碼</t>
+  </si>
+  <si>
+    <t>K987654(3)</t>
+  </si>
+  <si>
     <t>As shown on ID copy / 與身分證副本一致</t>
-  </si>
-  <si>
-    <t>contacts.0.title</t>
-  </si>
-  <si>
-    <t>Contact 1 / 聯絡人 1 - Title / 職位</t>
-  </si>
-  <si>
-    <t>Purchasing Manager</t>
-  </si>
-  <si>
-    <t>contacts.0.email</t>
-  </si>
-  <si>
-    <t>Contact 1 / 聯絡人 1 - Email / 電郵</t>
-  </si>
-  <si>
-    <t>john.wong@apex-trading-demo.hk</t>
-  </si>
-  <si>
-    <t>contacts.0.phoneCountryCode</t>
-  </si>
-  <si>
-    <t>Contact 1 / 聯絡人 1 - Phone Country Code / 電話區號</t>
-  </si>
-  <si>
-    <t>+852</t>
-  </si>
-  <si>
-    <t>e.g. +852</t>
-  </si>
-  <si>
-    <t>contacts.0.phone</t>
-  </si>
-  <si>
-    <t>Contact 1 / 聯絡人 1 - Phone / 電話</t>
-  </si>
-  <si>
-    <t>9123 4567</t>
-  </si>
-  <si>
-    <t>contacts.1.nameEnFirst</t>
-  </si>
-  <si>
-    <t>Contact 2 / 聯絡人 2 - Given Name (English) / 英文名 *</t>
-  </si>
-  <si>
-    <t>Mary</t>
-  </si>
-  <si>
-    <t>contacts.1.nameEnMiddle</t>
-  </si>
-  <si>
-    <t>Contact 2 / 聯絡人 2 - Middle Name (English) / 英文中間名</t>
-  </si>
-  <si>
-    <t>Ann</t>
-  </si>
-  <si>
-    <t>contacts.1.nameEnLast</t>
-  </si>
-  <si>
-    <t>Contact 2 / 聯絡人 2 - Surname (English) / 英文姓氏 *</t>
-  </si>
-  <si>
-    <t>Cheung</t>
-  </si>
-  <si>
-    <t>contacts.1.nameZh</t>
-  </si>
-  <si>
-    <t>Contact 2 / 聯絡人 2 - Full Name (Chinese) / 中文姓名全名 *</t>
-  </si>
-  <si>
-    <t>張麗珍</t>
-  </si>
-  <si>
-    <t>contacts.1.idNumber</t>
-  </si>
-  <si>
-    <t>Contact 2 / 聯絡人 2 - ID Number / 身分證號碼</t>
-  </si>
-  <si>
-    <t>K987654(3)</t>
   </si>
   <si>
     <t>contacts.1.title</t>
@@ -2620,18 +2623,18 @@
         <v>224</v>
       </c>
       <c r="D57" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B58" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C58" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D58" t="s">
         <v>32</v>
@@ -2639,13 +2642,13 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B59" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C59" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D59" t="s">
         <v>32</v>
@@ -2653,10 +2656,10 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B60" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C60" t="s">
         <v>205</v>
@@ -2667,13 +2670,13 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B61" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C61" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D61" t="s">
         <v>32</v>
@@ -2681,13 +2684,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B62" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C62" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D62" t="s">
         <v>32</v>
@@ -2695,10 +2698,10 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B63" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C63" t="s">
         <v>32</v>
@@ -2709,13 +2712,13 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B64" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C64" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D64" t="s">
         <v>32</v>
@@ -2723,13 +2726,13 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B65" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C65" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D65" t="s">
         <v>32</v>
@@ -2737,27 +2740,27 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B66" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C66" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D66" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B67" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C67" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D67" t="s">
         <v>32</v>
@@ -2765,13 +2768,13 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B68" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C68" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D68" t="s">
         <v>32</v>
@@ -2779,10 +2782,10 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B69" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C69" t="s">
         <v>205</v>
@@ -2793,13 +2796,13 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B70" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C70" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D70" t="s">
         <v>32</v>
@@ -2807,13 +2810,13 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B71" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C71" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D71" t="s">
         <v>32</v>
@@ -2821,10 +2824,10 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B72" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C72" t="s">
         <v>32</v>
@@ -2835,13 +2838,13 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B73" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C73" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D73" t="s">
         <v>32</v>
@@ -2849,13 +2852,13 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B74" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C74" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D74" t="s">
         <v>32</v>
@@ -2863,13 +2866,13 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B75" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C75" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D75" t="s">
         <v>32</v>
@@ -2877,13 +2880,13 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B76" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C76" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D76" t="s">
         <v>32</v>
@@ -2891,10 +2894,10 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B77" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C77" t="s">
         <v>205</v>
@@ -2905,13 +2908,13 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B78" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C78" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D78" t="s">
         <v>32</v>
@@ -2919,13 +2922,13 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B79" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C79" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D79" t="s">
         <v>32</v>
@@ -2933,10 +2936,10 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B80" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C80" t="s">
         <v>205</v>
@@ -2947,13 +2950,13 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B81" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C81" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D81" t="s">
         <v>32</v>
@@ -2961,30 +2964,30 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B82" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C82" t="s">
         <v>7</v>
       </c>
       <c r="D82" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B83" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C83" t="s">
         <v>11</v>
       </c>
       <c r="D83" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -2992,7 +2995,7 @@
         <v>32</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C84" t="s">
         <v>32</v>
@@ -3003,13 +3006,13 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B85" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C85" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D85" t="s">
         <v>32</v>
@@ -3017,13 +3020,13 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B86" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C86" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D86" t="s">
         <v>32</v>
@@ -3031,41 +3034,41 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B87" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C87" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D87" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B88" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C88" t="s">
         <v>76</v>
       </c>
       <c r="D88" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B89" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C89" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D89" t="s">
         <v>32</v>
@@ -3073,13 +3076,13 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B90" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C90" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D90" t="s">
         <v>32</v>

</xml_diff>